<commit_message>
M0-P10-1 10.2.12 docs(architecture): add strict per-file dependency graph with injections and lifecycle runbook
</commit_message>
<xml_diff>
--- a/docs/business/AVRAI_BUDGET.xlsx
+++ b/docs/business/AVRAI_BUDGET.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -603,370 +603,368 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>GitHub Pro</t>
+          <t>Cursor Bugbot (GitHub code checking)</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>48</v>
+        <v>480</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Private repos + GitHub Actions CI/CD</t>
+          <t>Automated PR/code checking integration through Cursor on GitHub.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>GitHub Pro</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Private repos + GitHub Actions CI/CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
           <t>Apple Developer Account</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B11" s="7" t="n">
         <v>8.25</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C11" s="7" t="n">
         <v>99</v>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>iOS distribution + TestFlight. $99/yr billed annually.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="9">
-        <f>SUM(B6:B10)</f>
+      <c r="B12" s="9">
+        <f>SUM(B6:B11)</f>
         <v/>
       </c>
-      <c r="C11" s="9">
-        <f>SUM(C6:C10)</f>
+      <c r="C12" s="9">
+        <f>SUM(C6:C11)</f>
         <v/>
       </c>
-      <c r="D11" s="8" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="D12" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>FIXED COSTS — One-Time Fees</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Google Play Developer</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B16" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>One-time. Required for Android distribution.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>FIXED COSTS — Hardware (One-Time, Buy as Needed)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>MacBook Pro (M3/M4)</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="n">
-        <v>1999</v>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>3499</v>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Required for iOS builds (Xcode/macOS only). Skip if already owned.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Mac Mini (CI server)</t>
+          <t>MacBook Pro (M3/M4)</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>599</v>
+        <v>1999</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>1299</v>
+        <v>3499</v>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Automated builds/tests. Skip if using GitHub Actions.</t>
+          <t>Required for iOS builds (Xcode/macOS only). Skip if already owned.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>External Monitor (27" 4K)</t>
+          <t>Mac Mini (CI server)</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>299</v>
+        <v>599</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>799</v>
+        <v>1299</v>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Skip if already owned.</t>
+          <t>Automated builds/tests. Skip if using GitHub Actions.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>External SSD (1-4TB)</t>
+          <t>External Monitor (27" 4K)</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>79</v>
+        <v>299</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>299</v>
+        <v>799</v>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Backups, ML model files, Xcode archives</t>
+          <t>Skip if already owned.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>USB-C Hub/Dock + Cables</t>
+          <t>External SSD (1-4TB)</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>350</v>
-      </c>
-      <c r="D23" s="5" t="inlineStr"/>
+        <v>299</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Backups, ML model files, Xcode archives</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>iPhone 15 Pro</t>
+          <t>USB-C Hub/Dock + Cables</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>999</v>
+        <v>99</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>1199</v>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Primary iOS test device. Tier 3 (full world model + SLM capable).</t>
-        </is>
-      </c>
+        <v>350</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>iPhone 14 (or older)</t>
+          <t>iPhone 15 Pro</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>500</v>
+        <v>999</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>799</v>
+        <v>1199</v>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Backward compatibility / Tier 2 testing. Refurbished OK.</t>
+          <t>Primary iOS test device. Tier 3 (full world model + SLM capable).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Google Pixel 8</t>
+          <t>iPhone 14 (or older)</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>549</v>
+        <v>500</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>699</v>
+        <v>799</v>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Primary Android test device. Stock Android baseline. Tier 2-3.</t>
+          <t>Backward compatibility / Tier 2 testing. Refurbished OK.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Google Pixel 8</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
+        <v>549</v>
+      </c>
+      <c r="C27" s="6" t="n">
         <v>699</v>
       </c>
-      <c r="C27" s="6" t="n">
-        <v>899</v>
-      </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Samsung One UI behaves differently for BLE, notifications, permissions. Refurb OK.</t>
+          <t>Primary Android test device. Stock Android baseline. Tier 2-3.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t>Samsung Galaxy S24</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>699</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>899</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Samsung One UI behaves differently for BLE, notifications, permissions. Refurb OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
           <t>Budget Android (~$150 range)</t>
         </is>
       </c>
-      <c r="B28" s="6" t="n">
+      <c r="B29" s="6" t="n">
         <v>149</v>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C29" s="6" t="n">
         <v>299</v>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>Low-end / Tier 0-1 performance testing. Real users have cheap phones.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B29" s="10">
-        <f>SUM(B19:B28)</f>
+      <c r="B30" s="10">
+        <f>SUM(B20:B29)</f>
         <v/>
       </c>
-      <c r="C29" s="10">
-        <f>SUM(C19:C28)</f>
+      <c r="C30" s="10">
+        <f>SUM(C20:C29)</f>
         <v/>
       </c>
-      <c r="D29" s="8" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="D30" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>VARIABLE COSTS — APIs &amp; Cloud Services</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Current Cost</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>What It Does</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Google Gemini API</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Powers AI chat via llm-chat-stream edge function</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Free tier: 1,000 req/day, 15 RPM. Paid: ~$1.25/1M input tokens. Gemini Flash cuts 75%.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Google Places API (New)</t>
+          <t>Google Gemini API</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
@@ -974,19 +972,19 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Text search, nearby search, place details for spot discovery</t>
+          <t>Powers AI chat via llm-chat-stream edge function</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>$200/mo free credit. $17/1K text searches. Credit covers ~11K searches/mo.</t>
+          <t>Free tier: 1,000 req/day, 15 RPM. Paid: ~$1.25/1M input tokens. Gemini Flash cuts 75%.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Google Maps SDK</t>
+          <t>Google Places API (New)</t>
         </is>
       </c>
       <c r="B35" s="6" t="n">
@@ -994,19 +992,19 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Renders native map view</t>
+          <t>Text search, nearby search, place details for spot discovery</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>$200/mo free credit shared with Places. $7/1K map loads.</t>
+          <t>$200/mo free credit. $17/1K text searches. Credit covers ~11K searches/mo.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Firebase (Blaze plan)</t>
+          <t>Google Maps SDK</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
@@ -1014,19 +1012,19 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Auth, Firestore, Storage (tax docs), Analytics (free), FCM push (free)</t>
+          <t>Renders native map view</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Free tier: 50K reads/day, 20K writes/day, 5GB storage.</t>
+          <t>$200/mo free credit shared with Places. $7/1K map loads.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>OpenWeatherMap</t>
+          <t>Firebase (Blaze plan)</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
@@ -1034,19 +1032,19 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Weather context for recommendations (indoor spots on rainy days)</t>
+          <t>Auth, Firestore, Storage (tax docs), Analytics (free), FCM push (free)</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Free tier: 1,000 calls/day. API key not yet configured.</t>
+          <t>Free tier: 50K reads/day, 20K writes/day, 5GB storage.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>OpenWeatherMap</t>
         </is>
       </c>
       <c r="B38" s="6" t="n">
@@ -1054,19 +1052,19 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Payments, refunds, identity verification</t>
+          <t>Weather context for recommendations (indoor spots on rainy days)</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>No monthly fee. 2.9% + $0.30/txn. $1.50/identity verification. Costs only when processing real money.</t>
+          <t>Free tier: 1,000 calls/day. API key not yet configured.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Google Cloud Storage</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="B39" s="6" t="n">
@@ -1074,19 +1072,19 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>File/media storage beyond Supabase</t>
+          <t>Payments, refunds, identity verification</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>5GB free. $0.020/GB/mo after.</t>
+          <t>No monthly fee. 2.9% + $0.30/txn. $1.50/identity verification. Costs only when processing real money.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Supabase Storage (model distribution)</t>
+          <t>Google Cloud Storage</t>
         </is>
       </c>
       <c r="B40" s="6" t="n">
@@ -1094,19 +1092,19 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>On-device ONNX models (~1MB) + optional SLM (700MB-2GB) downloaded by users</t>
+          <t>File/media storage beyond Supabase</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Included in Pro plan. Bandwidth = $0.09/GB egress. Migrate to Cloudflare R2 (free egress) before costs grow.</t>
+          <t>5GB free. $0.020/GB/mo after.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare R2 (future CDN)</t>
+          <t>Supabase Storage (model distribution)</t>
         </is>
       </c>
       <c r="B41" s="6" t="n">
@@ -1114,19 +1112,19 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Model delivery with free egress</t>
+          <t>On-device ONNX models (~1MB) + optional SLM (700MB-2GB) downloaded by users</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Not yet set up. $0.015/GB/mo storage. Use when model downloads create real bandwidth cost.</t>
+          <t>Included in Pro plan. Bandwidth = $0.09/GB egress. Migrate to Cloudflare R2 (free egress) before costs grow.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>ML Training Compute (Cloud GPU)</t>
+          <t>Cloudflare R2 (future CDN)</t>
         </is>
       </c>
       <c r="B42" s="6" t="n">
@@ -1134,283 +1132,439 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
+          <t>Model delivery with free egress</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Not yet set up. $0.015/GB/mo storage. Use when model downloads create real bandwidth cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ML Training Compute (Cloud GPU)</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
           <t>Pre-training energy function, transition predictor, batch retraining</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>Google Colab free tier for now. RunPod/Lambda $10-$50/run when needed.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>FREE SERVICES — No Budget Impact</t>
-        </is>
-      </c>
-    </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>PLANNED RESILIENCE/GOVERNANCE RESERVE (Master Plan 10.9.x + ML Governance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>What It Does</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Why Free</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>OpenStreetMap (Nominatim + Overpass)</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>Place search fallback, nearby amenity queries</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr"/>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Community API, free with rate limiting</t>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Monthly (Low)</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Monthly (High)</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Why It Exists</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Apple MapKit (MKLocalSearch)</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Native iOS place search with cache</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr"/>
+          <t>Observability + reliability tooling reserve</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>300</v>
+      </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Native SDK, no per-call cost</t>
+          <t>Dashboards/alerts and operational visibility for break-to-learning metrics (TTD, TTH, recurrence, impact radius).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Firebase Analytics</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Event tracking</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr"/>
+          <t>GitHub CI/check overage reserve</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>150</v>
+      </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Always free, unlimited</t>
+          <t>Additional required checks/workflow volume from execution + traceability + architecture + ML governance guards.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Firebase Cloud Messaging</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Push notifications</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr"/>
+          <t>ML retraining/simulation compute reserve</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>600</v>
+      </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Always free, unlimited</t>
+          <t>Non-free burst training/simulation runs and replay cycles as model scope expands.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Google OAuth</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Google Sign-In</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr"/>
+          <t>Data pipeline/storage/egress reserve</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>200</v>
+      </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Training artifacts, experiment logs, recovery queue growth, and transfer overhead.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Embeddings edge function</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>Text embeddings</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr"/>
+          <t>Contingency on resilience reserve (10-15%)</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>187.5</v>
+      </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Uses local hash, no external API</t>
+          <t>Buffer for reopen events and unexpected remediation loops.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>Social media OAuth (10 platforms)</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Instagram, Facebook, X, Reddit, TikTok, Pinterest, LinkedIn, YouTube, Tumblr, Are.na</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr"/>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>OAuth endpoints free. Behind feature flag.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>HuggingFace</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>Token configured, no active calls</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr"/>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Free tier</t>
-        </is>
-      </c>
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL RESILIENCE RESERVE ENVELOPE</t>
+        </is>
+      </c>
+      <c r="B52" s="9">
+        <f>SUM(B47:B51)</f>
+        <v/>
+      </c>
+      <c r="C52" s="9">
+        <f>SUM(C47:C51)</f>
+        <v/>
+      </c>
+      <c r="D52" s="8" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>TestFlight</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>iOS beta distribution</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr"/>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Included with Apple Developer</t>
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>FREE SERVICES — No Budget Impact</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Signal Protocol</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>End-to-end encryption for AI2AI</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr"/>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Runs entirely on-device (Rust FFI)</t>
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>What It Does</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Why Free</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>ONNX Runtime</t>
+          <t>OpenStreetMap (Nominatim + Overpass)</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>On-device world model inference (energy function, state encoder, transition predictor, action encoder)</t>
+          <t>Place search fallback, nearby amenity queries</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr"/>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Open-source, bundled in app binary</t>
+          <t>Community API, free with rate limiting</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>Drift / SQLite</t>
+          <t>Apple MapKit (MKLocalSearch)</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>On-device episodic memory, semantic memory storage</t>
+          <t>Native iOS place search with cache</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr"/>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Open-source, on-device</t>
+          <t>Native SDK, no per-call cost</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>PyTorch + ONNX tools</t>
+          <t>Firebase Analytics</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Training pipeline for world model components</t>
+          <t>Event tracking</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr"/>
       <c r="D58" s="5" t="inlineStr">
         <is>
+          <t>Always free, unlimited</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Firebase Cloud Messaging</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Push notifications</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr"/>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Always free, unlimited</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Google OAuth</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Google Sign-In</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr"/>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>Embeddings edge function</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Text embeddings</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr"/>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Uses local hash, no external API</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Social media OAuth (10 platforms)</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Instagram, Facebook, X, Reddit, TikTok, Pinterest, LinkedIn, YouTube, Tumblr, Are.na</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>OAuth endpoints free. Behind feature flag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>HuggingFace</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Token configured, no active calls</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr"/>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Free tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>TestFlight</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>iOS beta distribution</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr"/>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Included with Apple Developer</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Signal Protocol</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>End-to-end encryption for AI2AI</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr"/>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Runs entirely on-device (Rust FFI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>ONNX Runtime</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>On-device world model inference (energy function, state encoder, transition predictor, action encoder)</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr"/>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Open-source, bundled in app binary</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Drift / SQLite</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>On-device episodic memory, semantic memory storage</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr"/>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Open-source, on-device</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>PyTorch + ONNX tools</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Training pipeline for world model components</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr"/>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
           <t>Open-source Python libraries</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A18:D18"/>
     <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A54:D54"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2226,7 +2380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2325,357 +2479,427 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Cursor Bugbot (GitHub code checking)</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C9" s="5" t="n"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Admin, research, drafting</t>
+          <t>Automated PR/code checking integration through Cursor on GitHub</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>GitHub Pro</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Private repos + CI/CD</t>
+          <t>Admin, research, drafting</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>GitHub Pro</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C11" s="5" t="n"/>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>@avrai.org email ($3.50/mo promo through May '26)</t>
+          <t>Private repos + CI/CD</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Apple Developer (amortized)</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>8.25</v>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>$99/yr billed annually</t>
+          <t>@avrai.org email ($3.50/mo promo through May '26)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>All APIs &amp; Cloud Services</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>0</v>
+          <t>Apple Developer (amortized)</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>8.25</v>
       </c>
       <c r="C13" s="5" t="n"/>
       <c r="D13" s="5" t="inlineStr">
         <is>
+          <t>$99/yr billed annually</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>All APIs &amp; Cloud Services</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
           <t>All free tiers during solo development</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>TOTAL MONTHLY BURN</t>
         </is>
       </c>
-      <c r="B14" s="9">
-        <f>SUM(B6:B13)</f>
+      <c r="B15" s="9">
+        <f>SUM(B6:B14)</f>
         <v/>
       </c>
-      <c r="C14" s="10">
-        <f>B14*12</f>
+      <c r="C15" s="10">
+        <f>B15*12</f>
         <v/>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Per year</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>ONE-TIME COSTS — By Priority</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Resilience reserve envelope (low-high)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>214.5</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1437.5</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Master-plan 10.9.x + ML governance reserve</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>When</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Total monthly burn with reserve</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>4018.75</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>5241.75</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Committed burn + resilience reserve envelope</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Legal formation (2 LLCs + legal docs)</t>
+          <t>Total annual burn with reserve</t>
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>2390</v>
+        <v>48225</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>7990</v>
+        <v>62901</v>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Google Play Developer account</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Now</t>
+          <t>Annualized from monthly reserve-inclusive range</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Test devices (1-5 phones)</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>149</v>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>3895</v>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Before beta</t>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>ONE-TIME COSTS — By Priority</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>App designer (UI/UX + logo)</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n">
-        <v>3200</v>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>12000</v>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Before beta</t>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>When</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Development hardware (if needed)</t>
+          <t>Legal formation (2 LLCs + legal docs)</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>3075</v>
+        <v>2390</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>6246</v>
+        <v>7990</v>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>As needed — skip if already owned</t>
+          <t>Now</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Patent attorney + 5 provisionals</t>
+          <t>Google Play Developer account</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>12000</v>
+        <v>25</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>30000</v>
+        <v>25</v>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>When fundable</t>
+          <t>Now</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Security audit + legal compliance</t>
+          <t>Test devices (1-5 phones)</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>15000</v>
+        <v>149</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>35000</v>
+        <v>3895</v>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Post-raise</t>
+          <t>Before beta</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>App designer (UI/UX + logo)</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Before beta</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL CAPITAL NEEDED — Scenarios (Year 1)</t>
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Development hardware (if needed)</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>3075</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>6246</v>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>As needed — skip if already owned</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>One-Time</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Year 1 Burn</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Year 1 Total</t>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Patent attorney + 5 provisionals</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>When fundable</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t>Security audit + legal compliance</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>35000</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Post-raise</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL CAPITAL NEEDED — Scenarios (Year 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>One-Time</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Year 1 Burn</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Year 1 Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
           <t>Minimum viable (burn + LLCs + 1 phone)</t>
         </is>
       </c>
-      <c r="B28" s="6" t="n">
+      <c r="B32" s="6" t="n">
         <v>2564</v>
       </c>
-      <c r="C28" s="6" t="n">
-        <v>45171</v>
-      </c>
-      <c r="D28" s="6" t="n">
-        <v>47735</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="C32" s="6" t="n">
+        <v>45651</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>48215</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>Comfortable to beta (+ designer + phones + legal docs)</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n">
+      <c r="B33" s="6" t="n">
         <v>10860</v>
       </c>
-      <c r="C29" s="6" t="n">
-        <v>45171</v>
-      </c>
-      <c r="D29" s="6" t="n">
-        <v>56031</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="C33" s="6" t="n">
+        <v>45651</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>56511</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Full pre-seed (+ patents)</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n">
+      <c r="B34" s="6" t="n">
         <v>22860</v>
       </c>
-      <c r="C30" s="6" t="n">
-        <v>45171</v>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>68031</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="C34" s="6" t="n">
+        <v>45651</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>68511</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>Everything (+ security audit + all hardware)</t>
         </is>
       </c>
-      <c r="B31" s="6" t="n">
+      <c r="B35" s="6" t="n">
         <v>69306</v>
       </c>
-      <c r="C31" s="6" t="n">
-        <v>45171</v>
-      </c>
-      <c r="D31" s="6" t="n">
-        <v>114477</v>
+      <c r="C35" s="6" t="n">
+        <v>45651</v>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>114957</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A30:D30"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>